<commit_message>
chore(data-release): publish site data 2026-10-31 15:19:57 UTC
</commit_message>
<xml_diff>
--- a/diseases/d030/2010-2014.xlsx
+++ b/diseases/d030/2010-2014.xlsx
@@ -7809,9 +7809,9 @@
       <c r="R53" t="n">
         <v>0.0004931730985003484</v>
       </c>
-      <c r="AA53" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO53" t="inlineStr">
@@ -7821,12 +7821,22 @@
       </c>
       <c r="AP53" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR53" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS53" t="inlineStr"/>
       <c r="AT53" t="n">
         <v>0</v>
+      </c>
+      <c r="AU53" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
       </c>
       <c r="AV53" t="inlineStr">
         <is>
@@ -7944,9 +7954,9 @@
       <c r="R54" t="n">
         <v>0</v>
       </c>
-      <c r="AA54" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO54" t="inlineStr">
@@ -7956,13 +7966,23 @@
       </c>
       <c r="AP54" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR54" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS54" t="inlineStr"/>
       <c r="AT54" t="n">
         <v>0</v>
       </c>
+      <c r="AU54" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV54" t="inlineStr">
         <is>
           <t>all</t>
@@ -7973,6 +7993,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX54" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY54" t="inlineStr">
         <is>
           <t>web</t>
@@ -7988,7 +8013,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB54" t="inlineStr"/>
+      <c r="BB54" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC54" t="inlineStr">
         <is>
           <t>web</t>
@@ -8070,9 +8099,9 @@
       <c r="R55" t="n">
         <v>0</v>
       </c>
-      <c r="AA55" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO55" t="inlineStr">
@@ -8082,13 +8111,23 @@
       </c>
       <c r="AP55" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR55" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS55" t="inlineStr"/>
       <c r="AT55" t="n">
         <v>0</v>
       </c>
+      <c r="AU55" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV55" t="inlineStr">
         <is>
           <t>all</t>
@@ -8099,6 +8138,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX55" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY55" t="inlineStr">
         <is>
           <t>web</t>
@@ -8114,7 +8158,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB55" t="inlineStr"/>
+      <c r="BB55" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC55" t="inlineStr">
         <is>
           <t>web</t>
@@ -8196,9 +8244,9 @@
       <c r="R56" t="n">
         <v>0</v>
       </c>
-      <c r="AA56" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO56" t="inlineStr">
@@ -8208,13 +8256,23 @@
       </c>
       <c r="AP56" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR56" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS56" t="inlineStr"/>
       <c r="AT56" t="n">
         <v>0</v>
       </c>
+      <c r="AU56" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV56" t="inlineStr">
         <is>
           <t>all</t>
@@ -8225,6 +8283,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX56" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY56" t="inlineStr">
         <is>
           <t>web</t>
@@ -8240,7 +8303,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB56" t="inlineStr"/>
+      <c r="BB56" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC56" t="inlineStr">
         <is>
           <t>web</t>
@@ -8322,9 +8389,9 @@
       <c r="R57" t="n">
         <v>0</v>
       </c>
-      <c r="AA57" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO57" t="inlineStr">
@@ -8334,13 +8401,23 @@
       </c>
       <c r="AP57" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR57" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS57" t="inlineStr"/>
       <c r="AT57" t="n">
         <v>0</v>
       </c>
+      <c r="AU57" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV57" t="inlineStr">
         <is>
           <t>all</t>
@@ -8351,6 +8428,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX57" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY57" t="inlineStr">
         <is>
           <t>web</t>
@@ -8366,7 +8448,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB57" t="inlineStr"/>
+      <c r="BB57" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC57" t="inlineStr">
         <is>
           <t>web</t>
@@ -8448,9 +8534,9 @@
       <c r="R58" t="n">
         <v>0</v>
       </c>
-      <c r="AA58" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO58" t="inlineStr">
@@ -8460,13 +8546,23 @@
       </c>
       <c r="AP58" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR58" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS58" t="inlineStr"/>
       <c r="AT58" t="n">
         <v>0</v>
       </c>
+      <c r="AU58" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV58" t="inlineStr">
         <is>
           <t>all</t>
@@ -8477,6 +8573,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX58" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY58" t="inlineStr">
         <is>
           <t>web</t>
@@ -8492,7 +8593,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB58" t="inlineStr"/>
+      <c r="BB58" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC58" t="inlineStr">
         <is>
           <t>web</t>
@@ -8574,9 +8679,9 @@
       <c r="R59" t="n">
         <v>0</v>
       </c>
-      <c r="AA59" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO59" t="inlineStr">
@@ -8586,13 +8691,23 @@
       </c>
       <c r="AP59" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR59" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS59" t="inlineStr"/>
       <c r="AT59" t="n">
         <v>0</v>
       </c>
+      <c r="AU59" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV59" t="inlineStr">
         <is>
           <t>all</t>
@@ -8603,6 +8718,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX59" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY59" t="inlineStr">
         <is>
           <t>web</t>
@@ -8618,7 +8738,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB59" t="inlineStr"/>
+      <c r="BB59" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC59" t="inlineStr">
         <is>
           <t>web</t>
@@ -8700,9 +8824,9 @@
       <c r="R60" t="n">
         <v>0</v>
       </c>
-      <c r="AA60" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO60" t="inlineStr">
@@ -8712,13 +8836,23 @@
       </c>
       <c r="AP60" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR60" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS60" t="inlineStr"/>
       <c r="AT60" t="n">
         <v>0</v>
       </c>
+      <c r="AU60" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV60" t="inlineStr">
         <is>
           <t>all</t>
@@ -8729,6 +8863,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX60" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY60" t="inlineStr">
         <is>
           <t>web</t>
@@ -8744,7 +8883,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB60" t="inlineStr"/>
+      <c r="BB60" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC60" t="inlineStr">
         <is>
           <t>web</t>
@@ -8826,9 +8969,9 @@
       <c r="R61" t="n">
         <v>0</v>
       </c>
-      <c r="AA61" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO61" t="inlineStr">
@@ -8838,13 +8981,23 @@
       </c>
       <c r="AP61" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR61" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS61" t="inlineStr"/>
       <c r="AT61" t="n">
         <v>0</v>
       </c>
+      <c r="AU61" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV61" t="inlineStr">
         <is>
           <t>all</t>
@@ -8855,6 +9008,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX61" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY61" t="inlineStr">
         <is>
           <t>web</t>
@@ -8870,7 +9028,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB61" t="inlineStr"/>
+      <c r="BB61" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC61" t="inlineStr">
         <is>
           <t>web</t>
@@ -8952,9 +9114,9 @@
       <c r="R62" t="n">
         <v>0</v>
       </c>
-      <c r="AA62" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO62" t="inlineStr">
@@ -8964,13 +9126,23 @@
       </c>
       <c r="AP62" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR62" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS62" t="inlineStr"/>
       <c r="AT62" t="n">
         <v>0</v>
       </c>
+      <c r="AU62" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV62" t="inlineStr">
         <is>
           <t>all</t>
@@ -8981,6 +9153,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX62" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY62" t="inlineStr">
         <is>
           <t>web</t>
@@ -8996,7 +9173,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB62" t="inlineStr"/>
+      <c r="BB62" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC62" t="inlineStr">
         <is>
           <t>web</t>
@@ -9078,9 +9259,9 @@
       <c r="R63" t="n">
         <v>0</v>
       </c>
-      <c r="AA63" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO63" t="inlineStr">
@@ -9090,13 +9271,23 @@
       </c>
       <c r="AP63" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR63" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS63" t="inlineStr"/>
       <c r="AT63" t="n">
         <v>0</v>
       </c>
+      <c r="AU63" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV63" t="inlineStr">
         <is>
           <t>all</t>
@@ -9107,6 +9298,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX63" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY63" t="inlineStr">
         <is>
           <t>web</t>
@@ -9122,7 +9318,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB63" t="inlineStr"/>
+      <c r="BB63" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC63" t="inlineStr">
         <is>
           <t>web</t>
@@ -9204,9 +9404,9 @@
       <c r="R64" t="n">
         <v>0.004822973481796675</v>
       </c>
-      <c r="AA64" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO64" t="inlineStr">
@@ -9216,13 +9416,23 @@
       </c>
       <c r="AP64" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR64" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS64" t="inlineStr"/>
       <c r="AT64" t="n">
         <v>0</v>
       </c>
+      <c r="AU64" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV64" t="inlineStr">
         <is>
           <t>all</t>
@@ -9233,6 +9443,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX64" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY64" t="inlineStr">
         <is>
           <t>web</t>
@@ -9248,7 +9463,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB64" t="inlineStr"/>
+      <c r="BB64" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC64" t="inlineStr">
         <is>
           <t>web</t>
@@ -9330,9 +9549,9 @@
       <c r="R65" t="n">
         <v>0</v>
       </c>
-      <c r="AA65" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO65" t="inlineStr">
@@ -9342,13 +9561,23 @@
       </c>
       <c r="AP65" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR65" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS65" t="inlineStr"/>
       <c r="AT65" t="n">
         <v>0</v>
       </c>
+      <c r="AU65" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV65" t="inlineStr">
         <is>
           <t>all</t>
@@ -9359,6 +9588,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX65" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY65" t="inlineStr">
         <is>
           <t>web</t>
@@ -9374,7 +9608,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB65" t="inlineStr"/>
+      <c r="BB65" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC65" t="inlineStr">
         <is>
           <t>web</t>
@@ -9456,9 +9694,9 @@
       <c r="R66" t="n">
         <v>0</v>
       </c>
-      <c r="AA66" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO66" t="inlineStr">
@@ -9468,13 +9706,23 @@
       </c>
       <c r="AP66" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR66" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS66" t="inlineStr"/>
       <c r="AT66" t="n">
         <v>0</v>
       </c>
+      <c r="AU66" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV66" t="inlineStr">
         <is>
           <t>all</t>
@@ -9485,6 +9733,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX66" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY66" t="inlineStr">
         <is>
           <t>web</t>
@@ -9500,7 +9753,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB66" t="inlineStr"/>
+      <c r="BB66" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC66" t="inlineStr">
         <is>
           <t>web</t>
@@ -9582,9 +9839,9 @@
       <c r="R67" t="n">
         <v>0</v>
       </c>
-      <c r="AA67" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO67" t="inlineStr">
@@ -9594,13 +9851,23 @@
       </c>
       <c r="AP67" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR67" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS67" t="inlineStr"/>
       <c r="AT67" t="n">
         <v>0</v>
       </c>
+      <c r="AU67" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV67" t="inlineStr">
         <is>
           <t>all</t>
@@ -9611,6 +9878,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX67" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY67" t="inlineStr">
         <is>
           <t>web</t>
@@ -9626,7 +9898,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB67" t="inlineStr"/>
+      <c r="BB67" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC67" t="inlineStr">
         <is>
           <t>web</t>
@@ -9708,9 +9984,9 @@
       <c r="R68" t="n">
         <v>0</v>
       </c>
-      <c r="AA68" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO68" t="inlineStr">
@@ -9720,13 +9996,23 @@
       </c>
       <c r="AP68" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR68" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS68" t="inlineStr"/>
       <c r="AT68" t="n">
         <v>0</v>
       </c>
+      <c r="AU68" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV68" t="inlineStr">
         <is>
           <t>all</t>
@@ -9737,6 +10023,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX68" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY68" t="inlineStr">
         <is>
           <t>web</t>
@@ -9752,7 +10043,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB68" t="inlineStr"/>
+      <c r="BB68" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC68" t="inlineStr">
         <is>
           <t>web</t>
@@ -9834,9 +10129,9 @@
       <c r="R69" t="n">
         <v>0</v>
       </c>
-      <c r="AA69" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO69" t="inlineStr">
@@ -9846,13 +10141,23 @@
       </c>
       <c r="AP69" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR69" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS69" t="inlineStr"/>
       <c r="AT69" t="n">
         <v>0</v>
       </c>
+      <c r="AU69" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV69" t="inlineStr">
         <is>
           <t>all</t>
@@ -9863,6 +10168,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX69" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY69" t="inlineStr">
         <is>
           <t>web</t>
@@ -9878,7 +10188,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB69" t="inlineStr"/>
+      <c r="BB69" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC69" t="inlineStr">
         <is>
           <t>web</t>
@@ -9960,9 +10274,9 @@
       <c r="R70" t="n">
         <v>0</v>
       </c>
-      <c r="AA70" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO70" t="inlineStr">
@@ -9972,13 +10286,23 @@
       </c>
       <c r="AP70" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR70" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS70" t="inlineStr"/>
       <c r="AT70" t="n">
         <v>0</v>
       </c>
+      <c r="AU70" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV70" t="inlineStr">
         <is>
           <t>all</t>
@@ -9989,6 +10313,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX70" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY70" t="inlineStr">
         <is>
           <t>web</t>
@@ -10004,7 +10333,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB70" t="inlineStr"/>
+      <c r="BB70" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC70" t="inlineStr">
         <is>
           <t>web</t>
@@ -10086,9 +10419,9 @@
       <c r="R71" t="n">
         <v>0</v>
       </c>
-      <c r="AA71" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO71" t="inlineStr">
@@ -10098,13 +10431,23 @@
       </c>
       <c r="AP71" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR71" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS71" t="inlineStr"/>
       <c r="AT71" t="n">
         <v>0</v>
       </c>
+      <c r="AU71" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV71" t="inlineStr">
         <is>
           <t>all</t>
@@ -10115,6 +10458,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX71" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY71" t="inlineStr">
         <is>
           <t>web</t>
@@ -10130,7 +10478,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB71" t="inlineStr"/>
+      <c r="BB71" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC71" t="inlineStr">
         <is>
           <t>web</t>
@@ -10212,9 +10564,9 @@
       <c r="R72" t="n">
         <v>0</v>
       </c>
-      <c r="AA72" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO72" t="inlineStr">
@@ -10224,13 +10576,23 @@
       </c>
       <c r="AP72" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR72" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS72" t="inlineStr"/>
       <c r="AT72" t="n">
         <v>0</v>
       </c>
+      <c r="AU72" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV72" t="inlineStr">
         <is>
           <t>all</t>
@@ -10241,6 +10603,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX72" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY72" t="inlineStr">
         <is>
           <t>web</t>
@@ -10256,7 +10623,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB72" t="inlineStr"/>
+      <c r="BB72" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC72" t="inlineStr">
         <is>
           <t>web</t>
@@ -10338,9 +10709,9 @@
       <c r="R73" t="n">
         <v>0</v>
       </c>
-      <c r="AA73" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO73" t="inlineStr">
@@ -10350,13 +10721,23 @@
       </c>
       <c r="AP73" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR73" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS73" t="inlineStr"/>
       <c r="AT73" t="n">
         <v>0</v>
       </c>
+      <c r="AU73" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV73" t="inlineStr">
         <is>
           <t>all</t>
@@ -10367,6 +10748,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX73" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY73" t="inlineStr">
         <is>
           <t>web</t>
@@ -10382,7 +10768,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB73" t="inlineStr"/>
+      <c r="BB73" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC73" t="inlineStr">
         <is>
           <t>web</t>
@@ -10464,9 +10854,9 @@
       <c r="R74" t="n">
         <v>0</v>
       </c>
-      <c r="AA74" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO74" t="inlineStr">
@@ -10476,13 +10866,23 @@
       </c>
       <c r="AP74" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR74" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS74" t="inlineStr"/>
       <c r="AT74" t="n">
         <v>0</v>
       </c>
+      <c r="AU74" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV74" t="inlineStr">
         <is>
           <t>all</t>
@@ -10493,6 +10893,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX74" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY74" t="inlineStr">
         <is>
           <t>web</t>
@@ -10508,7 +10913,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB74" t="inlineStr"/>
+      <c r="BB74" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC74" t="inlineStr">
         <is>
           <t>web</t>
@@ -10590,9 +10999,9 @@
       <c r="R75" t="n">
         <v>0</v>
       </c>
-      <c r="AA75" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO75" t="inlineStr">
@@ -10602,13 +11011,23 @@
       </c>
       <c r="AP75" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR75" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS75" t="inlineStr"/>
       <c r="AT75" t="n">
         <v>0</v>
       </c>
+      <c r="AU75" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV75" t="inlineStr">
         <is>
           <t>all</t>
@@ -10619,6 +11038,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX75" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY75" t="inlineStr">
         <is>
           <t>web</t>
@@ -10634,7 +11058,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB75" t="inlineStr"/>
+      <c r="BB75" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC75" t="inlineStr">
         <is>
           <t>web</t>
@@ -10716,9 +11144,9 @@
       <c r="R76" t="n">
         <v>0</v>
       </c>
-      <c r="AA76" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO76" t="inlineStr">
@@ -10728,13 +11156,23 @@
       </c>
       <c r="AP76" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR76" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS76" t="inlineStr"/>
       <c r="AT76" t="n">
         <v>0</v>
       </c>
+      <c r="AU76" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV76" t="inlineStr">
         <is>
           <t>all</t>
@@ -10745,6 +11183,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX76" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY76" t="inlineStr">
         <is>
           <t>web</t>
@@ -10760,7 +11203,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB76" t="inlineStr"/>
+      <c r="BB76" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC76" t="inlineStr">
         <is>
           <t>web</t>
@@ -10842,9 +11289,9 @@
       <c r="R77" t="n">
         <v>0</v>
       </c>
-      <c r="AA77" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO77" t="inlineStr">
@@ -10854,13 +11301,23 @@
       </c>
       <c r="AP77" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR77" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS77" t="inlineStr"/>
       <c r="AT77" t="n">
         <v>0</v>
       </c>
+      <c r="AU77" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV77" t="inlineStr">
         <is>
           <t>all</t>
@@ -10871,6 +11328,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX77" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY77" t="inlineStr">
         <is>
           <t>web</t>
@@ -10886,7 +11348,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB77" t="inlineStr"/>
+      <c r="BB77" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC77" t="inlineStr">
         <is>
           <t>web</t>
@@ -10968,9 +11434,9 @@
       <c r="R78" t="n">
         <v>0</v>
       </c>
-      <c r="AA78" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO78" t="inlineStr">
@@ -10980,13 +11446,23 @@
       </c>
       <c r="AP78" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR78" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS78" t="inlineStr"/>
       <c r="AT78" t="n">
         <v>0</v>
       </c>
+      <c r="AU78" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV78" t="inlineStr">
         <is>
           <t>all</t>
@@ -10997,6 +11473,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX78" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY78" t="inlineStr">
         <is>
           <t>web</t>
@@ -11012,7 +11493,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB78" t="inlineStr"/>
+      <c r="BB78" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC78" t="inlineStr">
         <is>
           <t>web</t>
@@ -11094,9 +11579,9 @@
       <c r="R79" t="n">
         <v>0</v>
       </c>
-      <c r="AA79" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO79" t="inlineStr">
@@ -11106,13 +11591,23 @@
       </c>
       <c r="AP79" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR79" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS79" t="inlineStr"/>
       <c r="AT79" t="n">
         <v>0</v>
       </c>
+      <c r="AU79" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV79" t="inlineStr">
         <is>
           <t>all</t>
@@ -11123,6 +11618,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX79" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY79" t="inlineStr">
         <is>
           <t>web</t>
@@ -11138,7 +11638,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB79" t="inlineStr"/>
+      <c r="BB79" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC79" t="inlineStr">
         <is>
           <t>web</t>
@@ -11220,9 +11724,9 @@
       <c r="R80" t="n">
         <v>0</v>
       </c>
-      <c r="AA80" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>ibge_computed</t>
         </is>
       </c>
       <c r="AO80" t="inlineStr">
@@ -11232,13 +11736,23 @@
       </c>
       <c r="AP80" t="inlineStr">
         <is>
-          <t>published_series</t>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR80" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
         </is>
       </c>
       <c r="AS80" t="inlineStr"/>
       <c r="AT80" t="n">
         <v>0</v>
       </c>
+      <c r="AU80" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
       <c r="AV80" t="inlineStr">
         <is>
           <t>all</t>
@@ -11249,6 +11763,11 @@
           <t>All Sources</t>
         </is>
       </c>
+      <c r="AX80" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="AY80" t="inlineStr">
         <is>
           <t>web</t>
@@ -11264,7 +11783,11 @@
           <t>All Sources</t>
         </is>
       </c>
-      <c r="BB80" t="inlineStr"/>
+      <c r="BB80" t="inlineStr">
+        <is>
+          <t>http://siab.datasus.gov.br/DATASUS/index.php?acao=41&amp;area=0901&amp;item=1</t>
+        </is>
+      </c>
       <c r="BC80" t="inlineStr">
         <is>
           <t>web</t>

</xml_diff>